<commit_message>
Update Excel: add 8 SQL Injection cases (SEC08-SEC15)
Sync test case sheet with automation: the security sheet now has 12
SQLi cases (SEC01-04, SEC08-15), 2 XSS (SEC05-06), 1 DoS design (SEC07).
</commit_message>
<xml_diff>
--- a/testcases/TestCase_DangNhap_VanPhongDienTu.xlsx
+++ b/testcases/TestCase_DangNhap_VanPhongDienTu.xlsx
@@ -546,7 +546,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• BaoMat   : 7 test case bảo mật (SQLi, XSS, và mục DoS thiết kế-không-thực-thi).</t>
+          <t>• BaoMat   : 15 test case bảo mật — 12 SQL Injection (SEC01-04, SEC08-15), 2 XSS (SEC05-06), 1 DoS thiết kế-không-thực-thi (SEC07).</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1382,130 +1382,490 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
+          <t>SEC08</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Điều kiện luôn đúng kèm chú thích (OR 1=1--)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập payload vào username
+2. Nhập password bất kỳ
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>username = ' OR 1=1--
+password = x</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG bypass đăng nhập. Báo sai tài khoản.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>SEC09</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Chú thích kiểu MySQL (#) để bỏ qua kiểm tra mật khẩu</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập payload có '#' vào username
+2. Nhập password bất kỳ
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>username = admin'#
+password = x</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG bypass đăng nhập.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>SEC10</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>UNION-based: nối thêm câu lệnh SELECT</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập payload UNION SELECT vào username
+2. Nhập password bất kỳ
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>username = ' UNION SELECT 1,2,3--
+password = x</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG lộ dữ liệu, KHÔNG bypass. Báo sai tài khoản.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>SEC11</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>So sánh chuỗi rỗng bằng chuỗi rỗng (OR ''='')</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập payload vào username
+2. Nhập password bất kỳ
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>username = ' OR ''='
+password = x</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG bypass đăng nhập.</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>SEC12</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Thoát dấu ngoặc đơn/kép trong câu truy vấn</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập payload có dấu ngoặc vào username
+2. Nhập password bất kỳ
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>username = ") OR ("1"="1
+password = x</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG bypass đăng nhập.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>SEC13</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Payload ở ô mật khẩu dùng nháy kép</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập username hợp lệ
+2. Nhập payload vào password
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>username = student
+password = " OR ""="</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG bypass đăng nhập.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>SEC14</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Time-based blind: chèn lệnh trì hoãn (WAITFOR DELAY)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập payload WAITFOR DELAY vào username
+2. Nhập password bất kỳ
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>username = '; WAITFOR DELAY '0:0:5'--
+password = x</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG bị trì hoãn/treo, KHÔNG thực thi lệnh. Báo sai tài khoản ngay.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>SEC15</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>SQL Injection</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Stacked query: nối lệnh UPDATE đổi mật khẩu</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu là trang được phép kiểm thử</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>1. Nhập payload UPDATE vào username
+2. Nhập password bất kỳ
+3. Bấm Đăng nhập</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>username = x'; UPDATE users SET pass='1'--
+password = x</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG thực thi lệnh UPDATE, KHÔNG bypass. Báo sai tài khoản.</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>SEC05</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>XSS</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Chèn thẻ script vào ô username</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Mục tiêu là trang được phép kiểm thử</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>1. Nhập payload script vào username
 2. Nhập password bất kỳ
 3. Bấm Đăng nhập</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>username = &lt;script&gt;alert(1)&lt;/script&gt;
 password = x</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>KHÔNG xuất hiện hộp alert. Payload bị coi là chuỗi, không thực thi. Báo sai tài khoản.</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>SEC06</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>XSS</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Chèn thẻ img onerror (XSS qua thuộc tính sự kiện)</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Mục tiêu là trang được phép kiểm thử</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>1. Nhập payload img onerror vào username
 2. Bấm Đăng nhập</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>username = "&gt;&lt;img src=x onerror=alert(1)&gt;
 password = x</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>KHÔNG chạy mã JS, KHÔNG có alert. Hiển thị/đối xử như văn bản thuần.</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>SEC07</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>DoS / Tính sẵn sàng</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Tấn công từ chối dịch vụ (DoS/DDoS) — CHỈ THIẾT KẾ, KHÔNG THỰC THI tại đây</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>CẢNH BÁO: chỉ được chạy trên môi trường staging/được cấp phép bằng văn bản. TUYỆT ĐỐI không nhắm vào server thật vanphongdientu.utc.edu.vn.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Không cung cấp script tấn công. Nếu cần đánh giá tải: dùng công cụ load test (JMeter) trên môi trường được cấp phép, tăng tải dần có kiểm soát.</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>(không áp dụng)</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Biện pháp phòng thủ cần có: giới hạn tần suất (rate limiting), CAPTCHA sau nhiều lần sai, khoá tài khoản tạm thời, tường lửa ứng dụng web (WAF), chống tự động hoá. Hệ thống vẫn phục vụ người dùng hợp lệ khi bị quá tải.</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr"/>
-      <c r="J10" s="6" t="inlineStr"/>
+      <c r="I18" s="7" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>